<commit_message>
Model Sandefjord's fixed ice allocation as deterministic availability (issue #261)
Sandefjord Penguins is no longer treated as a required BookUp-scraped
calendar source. Their fixed weekend ice-time allocation (Sat/Sun
15:00-18:00 at Bugårdshallen, per the club's ISTIDER PLAN 26-27) is
now encoded in tournament_scheduler/sandefjord_allocation.py as
deterministic busy events and surfaced to Stage 2 as a new
"fixed_allocation" source type (pipeline/fixed_allocation_source.py),
so it flows through the existing sources -> events_by_club -> Stage 3
slot-search pipeline with no Sandefjord-specific planner code. Stage 2
never scrapes, blocks, or requires BookUp credentials for it; Tønsberg's
credentialed BookUp path is untouched. Removed the now-unused Sandefjord
scraper strategy and updated SKILL.md/README/docs accordingly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0128eSFqRwaCZeXoL3ScEWzh
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -3530,12 +3530,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>outlook</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>https://www.bookup.no/Utleie/#Bug%C3%A5rdshallen___/view:item/id:4497/part:/place:3907:SANDEFJORD/q:sandefjord/r:31/mod:book</t>
+          <t>fixed_allocation</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate season plan export from updated input.xlsx
Season window narrowed to 2026-10-09 start; re-ran the full RVV
pipeline (scrape -> plan -> export), resolving the JU12
Kongsberg/Tønsberg shared-host tie toward Tønsberg to balance
that registration's 3:1 hosting skew.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ATcxiMrpfz8cPn1rd3BLwH
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/niclasl/src/hockey/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{477B0544-71F0-5E4E-A657-DD1781C004EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B8A5CD8-AC79-DD45-97A8-5159B3686E98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38720" yWindow="-1640" windowWidth="26240" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="520" windowWidth="26240" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Innstillinger" sheetId="1" r:id="rId1"/>
@@ -34,9 +34,6 @@
     <t>start_date</t>
   </si>
   <si>
-    <t>2026-10-01</t>
-  </si>
-  <si>
     <t>end_date</t>
   </si>
   <si>
@@ -266,6 +263,9 @@
   </si>
   <si>
     <t>fixed_allocation</t>
+  </si>
+  <si>
+    <t>2026-10-09</t>
   </si>
 </sst>
 </file>
@@ -626,15 +626,15 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
         <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -654,24 +654,24 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>8</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>9</v>
-      </c>
-      <c r="E1" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2">
         <v>4</v>
@@ -688,7 +688,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3">
         <v>4</v>
@@ -705,7 +705,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4">
         <v>4</v>
@@ -722,7 +722,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5">
         <v>4</v>
@@ -739,7 +739,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6">
         <v>3</v>
@@ -756,7 +756,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7">
         <v>3</v>
@@ -773,7 +773,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B8">
         <v>3</v>
@@ -790,7 +790,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B9">
         <v>2</v>
@@ -807,7 +807,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B10">
         <v>2</v>
@@ -816,10 +816,10 @@
         <v>15</v>
       </c>
       <c r="D10">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E10">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -841,1575 +841,1575 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" t="s">
-        <v>21</v>
-      </c>
       <c r="C1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" t="s">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
-        <v>23</v>
-      </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" t="s">
         <v>26</v>
       </c>
-      <c r="B5" t="s">
-        <v>27</v>
-      </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
         <v>30</v>
       </c>
-      <c r="B8" t="s">
-        <v>31</v>
-      </c>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" t="s">
         <v>36</v>
       </c>
-      <c r="B13" t="s">
-        <v>37</v>
-      </c>
       <c r="C13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" t="s">
         <v>40</v>
       </c>
-      <c r="B16" t="s">
-        <v>41</v>
-      </c>
       <c r="C16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21" spans="1:3" collapsed="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>43</v>
+      </c>
+      <c r="B21" t="s">
         <v>44</v>
       </c>
-      <c r="B21" t="s">
-        <v>45</v>
-      </c>
       <c r="C21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" t="s">
         <v>22</v>
       </c>
-      <c r="B23" t="s">
-        <v>23</v>
-      </c>
       <c r="C23" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B25" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C25" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B26" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C26" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B27" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C27" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B28" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
+        <v>25</v>
+      </c>
+      <c r="B29" t="s">
         <v>26</v>
       </c>
-      <c r="B29" t="s">
-        <v>27</v>
-      </c>
       <c r="C29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B30" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C30" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B31" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" t="s">
         <v>30</v>
       </c>
-      <c r="B32" t="s">
-        <v>31</v>
-      </c>
       <c r="C32" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B33" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C33" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B34" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C34" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B35" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C35" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
         <v>36</v>
       </c>
-      <c r="B36" t="s">
-        <v>37</v>
-      </c>
       <c r="C36" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C37" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B38" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C38" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B39" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C39" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C40" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" t="s">
         <v>44</v>
       </c>
-      <c r="B41" t="s">
-        <v>45</v>
-      </c>
       <c r="C41" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C42" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
+        <v>39</v>
+      </c>
+      <c r="B43" t="s">
         <v>40</v>
       </c>
-      <c r="B43" t="s">
-        <v>41</v>
-      </c>
       <c r="C43" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C44" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B45" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C45" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
+        <v>21</v>
+      </c>
+      <c r="B46" t="s">
         <v>22</v>
       </c>
-      <c r="B46" t="s">
-        <v>23</v>
-      </c>
       <c r="C46" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B47" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C47" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B48" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C48" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B49" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C49" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
+        <v>25</v>
+      </c>
+      <c r="B50" t="s">
         <v>26</v>
       </c>
-      <c r="B50" t="s">
-        <v>27</v>
-      </c>
       <c r="C50" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B51" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C51" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B52" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C52" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
+        <v>29</v>
+      </c>
+      <c r="B53" t="s">
         <v>30</v>
       </c>
-      <c r="B53" t="s">
-        <v>31</v>
-      </c>
       <c r="C53" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B54" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C54" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B55" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C55" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
+        <v>35</v>
+      </c>
+      <c r="B56" t="s">
         <v>36</v>
       </c>
-      <c r="B56" t="s">
-        <v>37</v>
-      </c>
       <c r="C56" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B57" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C57" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B58" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C58" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B59" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C59" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
+        <v>43</v>
+      </c>
+      <c r="B60" t="s">
         <v>44</v>
       </c>
-      <c r="B60" t="s">
-        <v>45</v>
-      </c>
       <c r="C60" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
+        <v>39</v>
+      </c>
+      <c r="B61" t="s">
         <v>40</v>
       </c>
-      <c r="B61" t="s">
-        <v>41</v>
-      </c>
       <c r="C61" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B62" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C62" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B63" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C63" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B64" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C64" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B65" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C65" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
+        <v>29</v>
+      </c>
+      <c r="B66" t="s">
         <v>30</v>
       </c>
-      <c r="B66" t="s">
-        <v>31</v>
-      </c>
       <c r="C66" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B67" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C67" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B68" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C68" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
+        <v>43</v>
+      </c>
+      <c r="B69" t="s">
         <v>44</v>
       </c>
-      <c r="B69" t="s">
-        <v>45</v>
-      </c>
       <c r="C69" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B70" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C70" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
+        <v>21</v>
+      </c>
+      <c r="B71" t="s">
         <v>22</v>
       </c>
-      <c r="B71" t="s">
-        <v>23</v>
-      </c>
       <c r="C71" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B72" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C72" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B73" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C73" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B74" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C74" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B75" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C75" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B76" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C76" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B77" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C77" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
+        <v>25</v>
+      </c>
+      <c r="B78" t="s">
         <v>26</v>
       </c>
-      <c r="B78" t="s">
-        <v>27</v>
-      </c>
       <c r="C78" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B79" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C79" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B80" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C80" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
+        <v>29</v>
+      </c>
+      <c r="B81" t="s">
         <v>30</v>
       </c>
-      <c r="B81" t="s">
-        <v>31</v>
-      </c>
       <c r="C81" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B82" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C82" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B83" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C83" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B84" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C84" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B85" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C85" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B86" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C86" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
+        <v>35</v>
+      </c>
+      <c r="B87" t="s">
         <v>36</v>
       </c>
-      <c r="B87" t="s">
-        <v>37</v>
-      </c>
       <c r="C87" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B88" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C88" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B89" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C89" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B90" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C90" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
+        <v>43</v>
+      </c>
+      <c r="B91" t="s">
         <v>44</v>
       </c>
-      <c r="B91" t="s">
-        <v>45</v>
-      </c>
       <c r="C91" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B92" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C92" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B93" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C93" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B94" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C94" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B95" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C95" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
+        <v>21</v>
+      </c>
+      <c r="B96" t="s">
         <v>22</v>
       </c>
-      <c r="B96" t="s">
-        <v>23</v>
-      </c>
       <c r="C96" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B97" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C97" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B98" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C98" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B99" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C99" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
+        <v>25</v>
+      </c>
+      <c r="B100" t="s">
         <v>26</v>
       </c>
-      <c r="B100" t="s">
-        <v>27</v>
-      </c>
       <c r="C100" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B101" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C101" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
+        <v>29</v>
+      </c>
+      <c r="B102" t="s">
         <v>30</v>
       </c>
-      <c r="B102" t="s">
-        <v>31</v>
-      </c>
       <c r="C102" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B103" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C103" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B104" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C104" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B105" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C105" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B106" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C106" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B107" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C107" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B108" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C108" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B109" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C109" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
+        <v>35</v>
+      </c>
+      <c r="B110" t="s">
         <v>36</v>
       </c>
-      <c r="B110" t="s">
-        <v>37</v>
-      </c>
       <c r="C110" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B111" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C111" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B112" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C112" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
+        <v>43</v>
+      </c>
+      <c r="B113" t="s">
         <v>44</v>
       </c>
-      <c r="B113" t="s">
-        <v>45</v>
-      </c>
       <c r="C113" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B114" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C114" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
+        <v>39</v>
+      </c>
+      <c r="B115" t="s">
         <v>40</v>
       </c>
-      <c r="B115" t="s">
-        <v>41</v>
-      </c>
       <c r="C115" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B116" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C116" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B117" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C117" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B118" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C118" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B119" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C119" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B120" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C120" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B121" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C121" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B122" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C122" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B123" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C123" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
+        <v>43</v>
+      </c>
+      <c r="B124" t="s">
         <v>44</v>
       </c>
-      <c r="B124" t="s">
-        <v>45</v>
-      </c>
       <c r="C124" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B125" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C125" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B126" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C126" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
+        <v>21</v>
+      </c>
+      <c r="B127" t="s">
         <v>22</v>
       </c>
-      <c r="B127" t="s">
-        <v>23</v>
-      </c>
       <c r="C127" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B128" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C128" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B129" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C129" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
+        <v>25</v>
+      </c>
+      <c r="B130" t="s">
         <v>26</v>
       </c>
-      <c r="B130" t="s">
-        <v>27</v>
-      </c>
       <c r="C130" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B131" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C131" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
+        <v>29</v>
+      </c>
+      <c r="B132" t="s">
         <v>30</v>
       </c>
-      <c r="B132" t="s">
-        <v>31</v>
-      </c>
       <c r="C132" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B133" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C133" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B134" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C134" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B135" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C135" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
+        <v>35</v>
+      </c>
+      <c r="B136" t="s">
         <v>36</v>
       </c>
-      <c r="B136" t="s">
-        <v>37</v>
-      </c>
       <c r="C136" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B137" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C137" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B138" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C138" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
+        <v>43</v>
+      </c>
+      <c r="B139" t="s">
         <v>44</v>
       </c>
-      <c r="B139" t="s">
-        <v>45</v>
-      </c>
       <c r="C139" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B140" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C140" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B141" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C141" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B142" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C142" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B143" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C143" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -2429,109 +2429,109 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B1" t="s">
         <v>66</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>67</v>
-      </c>
-      <c r="C1" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" t="s">
         <v>69</v>
-      </c>
-      <c r="C2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" t="s">
         <v>72</v>
-      </c>
-      <c r="C4" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" t="s">
         <v>79</v>
-      </c>
-      <c r="B10" t="s">
-        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>